<commit_message>
Uploading project's hybrid framework
</commit_message>
<xml_diff>
--- a/src/test/resources/TestData/SearchData.xlsx
+++ b/src/test/resources/TestData/SearchData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="12270" windowHeight="6800"/>
+    <workbookView windowWidth="18350" windowHeight="6800"/>
   </bookViews>
   <sheets>
     <sheet name="SearchData" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Product</t>
   </si>
@@ -45,6 +45,15 @@
   </si>
   <si>
     <t>Camera</t>
+  </si>
+  <si>
+    <t>Lap</t>
+  </si>
+  <si>
+    <t>xyz</t>
+  </si>
+  <si>
+    <t>$%@&amp;</t>
   </si>
 </sst>
 </file>
@@ -1197,8 +1206,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:A6"/>
-  <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5" outlineLevelRow="5"/>
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultColWidth="9.81818181818182" defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="13.1818181818182" customWidth="1"/>
   </cols>
@@ -1233,6 +1242,21 @@
         <v>5</v>
       </c>
     </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>